<commit_message>
Auto-zoom map to filtered sites; clean 6 mis-geocoded records
Map:
- When any filter is active, map auto-zooms and re-centers to the bounding
  box of matching sites (with 50% padding). Single county zooms to ~8.1,
  multi-county regional filter to ~7, all sites defaults to 5.5.
- Coordinates clamped to Texas bounds before bbox calc to guard against
  any future geocoding outliers.

Data quality:
- Removed 6 sites whose Google Places coordinates placed them outside Texas
  (Karnes, Medina, Crockett, Sterling, Duval, Live Oak counties each had
  one record geocoded to NM/OH/TN/KY/FL). Catalog: 639 -> 633 sites.
- Rebuilt food_access_county.xlsx to reflect corrected site counts.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/food_access_county.xlsx
+++ b/food_access_county.xlsx
@@ -133,6 +133,9 @@
     <t>Coke</t>
   </si>
   <si>
+    <t>Duval</t>
+  </si>
+  <si>
     <t>Willacy</t>
   </si>
   <si>
@@ -142,15 +145,15 @@
     <t>Real</t>
   </si>
   <si>
+    <t>La Salle</t>
+  </si>
+  <si>
     <t>Live Oak</t>
   </si>
   <si>
     <t>Maverick</t>
   </si>
   <si>
-    <t>La Salle</t>
-  </si>
-  <si>
     <t>Starr</t>
   </si>
   <si>
@@ -163,72 +166,69 @@
     <t>Bexar</t>
   </si>
   <si>
+    <t>Atascosa</t>
+  </si>
+  <si>
+    <t>Aransas</t>
+  </si>
+  <si>
+    <t>Lavaca</t>
+  </si>
+  <si>
+    <t>Sterling</t>
+  </si>
+  <si>
+    <t>Webb</t>
+  </si>
+  <si>
+    <t>Burnet</t>
+  </si>
+  <si>
+    <t>Crockett</t>
+  </si>
+  <si>
     <t>Sutton</t>
   </si>
   <si>
-    <t>Atascosa</t>
-  </si>
-  <si>
-    <t>Aransas</t>
-  </si>
-  <si>
-    <t>Lavaca</t>
-  </si>
-  <si>
-    <t>Sterling</t>
-  </si>
-  <si>
-    <t>Webb</t>
-  </si>
-  <si>
-    <t>Crockett</t>
+    <t>Colorado</t>
+  </si>
+  <si>
+    <t>Menard</t>
+  </si>
+  <si>
+    <t>Upton</t>
+  </si>
+  <si>
+    <t>Jim Wells</t>
+  </si>
+  <si>
+    <t>Irion</t>
+  </si>
+  <si>
+    <t>Matagorda</t>
+  </si>
+  <si>
+    <t>Mason</t>
+  </si>
+  <si>
+    <t>Calhoun</t>
+  </si>
+  <si>
+    <t>Goliad</t>
+  </si>
+  <si>
+    <t>Gonzales</t>
+  </si>
+  <si>
+    <t>Kinney</t>
+  </si>
+  <si>
+    <t>Cameron</t>
   </si>
   <si>
     <t>Concho</t>
   </si>
   <si>
-    <t>Burnet</t>
-  </si>
-  <si>
-    <t>Colorado</t>
-  </si>
-  <si>
-    <t>Menard</t>
-  </si>
-  <si>
-    <t>Upton</t>
-  </si>
-  <si>
-    <t>Jim Wells</t>
-  </si>
-  <si>
-    <t>Irion</t>
-  </si>
-  <si>
-    <t>Matagorda</t>
-  </si>
-  <si>
-    <t>Mason</t>
-  </si>
-  <si>
-    <t>Calhoun</t>
-  </si>
-  <si>
-    <t>Goliad</t>
-  </si>
-  <si>
-    <t>Gonzales</t>
-  </si>
-  <si>
-    <t>Kinney</t>
-  </si>
-  <si>
-    <t>Cameron</t>
-  </si>
-  <si>
-    <t>Duval</t>
-  </si>
-  <si>
     <t>Hays</t>
   </si>
   <si>
@@ -370,6 +370,9 @@
     <t>48081</t>
   </si>
   <si>
+    <t>48131</t>
+  </si>
+  <si>
     <t>48489</t>
   </si>
   <si>
@@ -379,15 +382,15 @@
     <t>48385</t>
   </si>
   <si>
+    <t>48283</t>
+  </si>
+  <si>
     <t>48297</t>
   </si>
   <si>
     <t>48323</t>
   </si>
   <si>
-    <t>48283</t>
-  </si>
-  <si>
     <t>48427</t>
   </si>
   <si>
@@ -400,72 +403,69 @@
     <t>48029</t>
   </si>
   <si>
+    <t>48013</t>
+  </si>
+  <si>
+    <t>48007</t>
+  </si>
+  <si>
+    <t>48285</t>
+  </si>
+  <si>
+    <t>48431</t>
+  </si>
+  <si>
+    <t>48479</t>
+  </si>
+  <si>
+    <t>48053</t>
+  </si>
+  <si>
+    <t>48105</t>
+  </si>
+  <si>
     <t>48435</t>
   </si>
   <si>
-    <t>48013</t>
-  </si>
-  <si>
-    <t>48007</t>
-  </si>
-  <si>
-    <t>48285</t>
-  </si>
-  <si>
-    <t>48431</t>
-  </si>
-  <si>
-    <t>48479</t>
-  </si>
-  <si>
-    <t>48105</t>
+    <t>48089</t>
+  </si>
+  <si>
+    <t>48327</t>
+  </si>
+  <si>
+    <t>48461</t>
+  </si>
+  <si>
+    <t>48249</t>
+  </si>
+  <si>
+    <t>48235</t>
+  </si>
+  <si>
+    <t>48321</t>
+  </si>
+  <si>
+    <t>48319</t>
+  </si>
+  <si>
+    <t>48057</t>
+  </si>
+  <si>
+    <t>48175</t>
+  </si>
+  <si>
+    <t>48177</t>
+  </si>
+  <si>
+    <t>48271</t>
+  </si>
+  <si>
+    <t>48061</t>
   </si>
   <si>
     <t>48095</t>
   </si>
   <si>
-    <t>48053</t>
-  </si>
-  <si>
-    <t>48089</t>
-  </si>
-  <si>
-    <t>48327</t>
-  </si>
-  <si>
-    <t>48461</t>
-  </si>
-  <si>
-    <t>48249</t>
-  </si>
-  <si>
-    <t>48235</t>
-  </si>
-  <si>
-    <t>48321</t>
-  </si>
-  <si>
-    <t>48319</t>
-  </si>
-  <si>
-    <t>48057</t>
-  </si>
-  <si>
-    <t>48175</t>
-  </si>
-  <si>
-    <t>48177</t>
-  </si>
-  <si>
-    <t>48271</t>
-  </si>
-  <si>
-    <t>48061</t>
-  </si>
-  <si>
-    <t>48131</t>
-  </si>
-  <si>
     <t>48209</t>
   </si>
   <si>
@@ -592,6 +592,9 @@
     <t>500</t>
   </si>
   <si>
+    <t>1850</t>
+  </si>
+  <si>
     <t>3960</t>
   </si>
   <si>
@@ -601,15 +604,15 @@
     <t>610</t>
   </si>
   <si>
+    <t>990</t>
+  </si>
+  <si>
     <t>1820</t>
   </si>
   <si>
     <t>11270</t>
   </si>
   <si>
-    <t>990</t>
-  </si>
-  <si>
     <t>15550</t>
   </si>
   <si>
@@ -622,66 +625,63 @@
     <t>278860</t>
   </si>
   <si>
+    <t>5740</t>
+  </si>
+  <si>
+    <t>4320</t>
+  </si>
+  <si>
+    <t>2460</t>
+  </si>
+  <si>
+    <t>110</t>
+  </si>
+  <si>
+    <t>42720</t>
+  </si>
+  <si>
+    <t>5560</t>
+  </si>
+  <si>
+    <t>340</t>
+  </si>
+  <si>
     <t>460</t>
   </si>
   <si>
-    <t>5740</t>
-  </si>
-  <si>
-    <t>4320</t>
-  </si>
-  <si>
-    <t>2460</t>
-  </si>
-  <si>
-    <t>110</t>
-  </si>
-  <si>
-    <t>42720</t>
-  </si>
-  <si>
-    <t>340</t>
+    <t>2050</t>
+  </si>
+  <si>
+    <t>420</t>
+  </si>
+  <si>
+    <t>7010</t>
+  </si>
+  <si>
+    <t>210</t>
+  </si>
+  <si>
+    <t>6320</t>
+  </si>
+  <si>
+    <t>2520</t>
+  </si>
+  <si>
+    <t>970</t>
+  </si>
+  <si>
+    <t>2620</t>
+  </si>
+  <si>
+    <t>620</t>
+  </si>
+  <si>
+    <t>75650</t>
   </si>
   <si>
     <t>430</t>
   </si>
   <si>
-    <t>5560</t>
-  </si>
-  <si>
-    <t>2050</t>
-  </si>
-  <si>
-    <t>420</t>
-  </si>
-  <si>
-    <t>7010</t>
-  </si>
-  <si>
-    <t>210</t>
-  </si>
-  <si>
-    <t>6320</t>
-  </si>
-  <si>
-    <t>2520</t>
-  </si>
-  <si>
-    <t>970</t>
-  </si>
-  <si>
-    <t>2620</t>
-  </si>
-  <si>
-    <t>620</t>
-  </si>
-  <si>
-    <t>75650</t>
-  </si>
-  <si>
-    <t>1850</t>
-  </si>
-  <si>
     <t>27620</t>
   </si>
   <si>
@@ -802,6 +802,9 @@
     <t>3.9</t>
   </si>
   <si>
+    <t>5.5</t>
+  </si>
+  <si>
     <t>4</t>
   </si>
   <si>
@@ -811,12 +814,12 @@
     <t>1.3</t>
   </si>
   <si>
+    <t>6.6</t>
+  </si>
+  <si>
     <t>7.1</t>
   </si>
   <si>
-    <t>6.6</t>
-  </si>
-  <si>
     <t>3.3</t>
   </si>
   <si>
@@ -872,9 +875,6 @@
   </si>
   <si>
     <t>5.1</t>
-  </si>
-  <si>
-    <t>5.5</t>
   </si>
   <si>
     <t>2.6</t>
@@ -1925,13 +1925,13 @@
         <v>39</v>
       </c>
       <c r="B9">
-        <v>4124</v>
+        <v>2561</v>
       </c>
       <c r="C9">
-        <v>1925</v>
+        <v>1271</v>
       </c>
       <c r="D9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -1952,7 +1952,7 @@
         <v>0</v>
       </c>
       <c r="K9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L9">
         <v>0</v>
@@ -1964,10 +1964,10 @@
         <v>100</v>
       </c>
       <c r="O9">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="P9">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="Q9">
         <v>11</v>
@@ -1976,10 +1976,10 @@
         <v>109</v>
       </c>
       <c r="S9">
-        <v>2062</v>
+        <v>2561</v>
       </c>
       <c r="T9">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="U9" t="b">
         <v>0</v>
@@ -1988,13 +1988,13 @@
         <v>1</v>
       </c>
       <c r="W9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X9" t="s">
         <v>118</v>
       </c>
       <c r="Y9">
-        <v>0.194</v>
+        <v>0.185</v>
       </c>
       <c r="Z9" t="s">
         <v>192</v>
@@ -2003,19 +2003,19 @@
         <v>262</v>
       </c>
       <c r="AB9">
-        <v>30.6606068387877</v>
+        <v>24.1636296257439</v>
       </c>
       <c r="AC9">
-        <v>36683.6</v>
+        <v>46913.66666666666</v>
       </c>
       <c r="AD9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AE9">
-        <v>19.4</v>
+        <v>18.5</v>
       </c>
       <c r="AF9">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:32">
@@ -2023,13 +2023,13 @@
         <v>40</v>
       </c>
       <c r="B10">
-        <v>1954</v>
+        <v>4124</v>
       </c>
       <c r="C10">
-        <v>929</v>
+        <v>1925</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -2050,22 +2050,22 @@
         <v>0</v>
       </c>
       <c r="K10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M10">
         <v>100</v>
       </c>
       <c r="N10">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O10">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="P10">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="Q10">
         <v>11</v>
@@ -2074,10 +2074,10 @@
         <v>109</v>
       </c>
       <c r="S10">
-        <v>1954</v>
+        <v>2062</v>
       </c>
       <c r="T10">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="U10" t="b">
         <v>0</v>
@@ -2086,13 +2086,13 @@
         <v>1</v>
       </c>
       <c r="W10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X10" t="s">
         <v>119</v>
       </c>
       <c r="Y10">
-        <v>0.233</v>
+        <v>0.194</v>
       </c>
       <c r="Z10" t="s">
         <v>193</v>
@@ -2101,16 +2101,16 @@
         <v>263</v>
       </c>
       <c r="AB10">
-        <v>37.12217510644845</v>
+        <v>30.6606068387877</v>
       </c>
       <c r="AC10">
-        <v>29893</v>
+        <v>36683.6</v>
       </c>
       <c r="AD10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AE10">
-        <v>23.3</v>
+        <v>19.4</v>
       </c>
       <c r="AF10">
         <v>6</v>
@@ -2121,10 +2121,10 @@
         <v>41</v>
       </c>
       <c r="B11">
-        <v>332</v>
+        <v>1954</v>
       </c>
       <c r="C11">
-        <v>164</v>
+        <v>929</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -2136,7 +2136,7 @@
         <v>0</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11">
         <v>0</v>
@@ -2151,28 +2151,28 @@
         <v>0</v>
       </c>
       <c r="L11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M11">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="N11">
         <v>0</v>
       </c>
       <c r="O11">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P11">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q11">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="R11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="S11">
-        <v>332</v>
+        <v>1954</v>
       </c>
       <c r="T11">
         <v>0</v>
@@ -2190,7 +2190,7 @@
         <v>120</v>
       </c>
       <c r="Y11">
-        <v>0.213</v>
+        <v>0.233</v>
       </c>
       <c r="Z11" t="s">
         <v>194</v>
@@ -2199,16 +2199,16 @@
         <v>264</v>
       </c>
       <c r="AB11">
-        <v>22.812879708384</v>
+        <v>37.12217510644845</v>
       </c>
       <c r="AC11">
-        <v>50000</v>
+        <v>29893</v>
       </c>
       <c r="AD11">
         <v>1</v>
       </c>
       <c r="AE11">
-        <v>21.3</v>
+        <v>23.3</v>
       </c>
       <c r="AF11">
         <v>6</v>
@@ -2219,22 +2219,22 @@
         <v>42</v>
       </c>
       <c r="B12">
-        <v>1229</v>
+        <v>332</v>
       </c>
       <c r="C12">
-        <v>571</v>
+        <v>164</v>
       </c>
       <c r="D12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12">
         <v>0</v>
@@ -2249,28 +2249,28 @@
         <v>0</v>
       </c>
       <c r="L12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M12">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="N12">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="O12">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="P12">
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="Q12">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="R12" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="S12">
-        <v>614</v>
+        <v>332</v>
       </c>
       <c r="T12">
         <v>0</v>
@@ -2288,7 +2288,7 @@
         <v>121</v>
       </c>
       <c r="Y12">
-        <v>0.16</v>
+        <v>0.213</v>
       </c>
       <c r="Z12" t="s">
         <v>195</v>
@@ -2297,19 +2297,19 @@
         <v>265</v>
       </c>
       <c r="AB12">
-        <v>15.7951107363978</v>
+        <v>22.812879708384</v>
       </c>
       <c r="AC12">
-        <v>60481</v>
+        <v>50000</v>
       </c>
       <c r="AD12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE12">
-        <v>16</v>
+        <v>21.3</v>
       </c>
       <c r="AF12">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:32">
@@ -2317,13 +2317,13 @@
         <v>43</v>
       </c>
       <c r="B13">
-        <v>15337</v>
+        <v>1082</v>
       </c>
       <c r="C13">
-        <v>6621</v>
+        <v>506</v>
       </c>
       <c r="D13">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E13">
         <v>0</v>
@@ -2332,7 +2332,7 @@
         <v>0</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H13">
         <v>0</v>
@@ -2347,19 +2347,19 @@
         <v>0</v>
       </c>
       <c r="L13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M13">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="N13">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="O13">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="P13">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="Q13">
         <v>8</v>
@@ -2368,7 +2368,7 @@
         <v>108</v>
       </c>
       <c r="S13">
-        <v>3834</v>
+        <v>1082</v>
       </c>
       <c r="T13">
         <v>0</v>
@@ -2386,25 +2386,25 @@
         <v>122</v>
       </c>
       <c r="Y13">
-        <v>0.195</v>
+        <v>0.143</v>
       </c>
       <c r="Z13" t="s">
         <v>196</v>
       </c>
       <c r="AA13" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="AB13">
-        <v>26.65128595503306</v>
+        <v>12.1464997681966</v>
       </c>
       <c r="AC13">
-        <v>42852.77777777778</v>
+        <v>53699</v>
       </c>
       <c r="AD13">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AE13">
-        <v>19.5</v>
+        <v>14.3</v>
       </c>
       <c r="AF13">
         <v>5</v>
@@ -2415,22 +2415,22 @@
         <v>44</v>
       </c>
       <c r="B14">
-        <v>1082</v>
+        <v>1229</v>
       </c>
       <c r="C14">
-        <v>506</v>
+        <v>571</v>
       </c>
       <c r="D14">
         <v>1</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14">
         <v>0</v>
       </c>
       <c r="G14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H14">
         <v>0</v>
@@ -2445,28 +2445,28 @@
         <v>0</v>
       </c>
       <c r="L14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M14">
         <v>100</v>
       </c>
       <c r="N14">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O14">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="P14">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q14">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="R14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="S14">
-        <v>1082</v>
+        <v>1229</v>
       </c>
       <c r="T14">
         <v>0</v>
@@ -2484,25 +2484,25 @@
         <v>123</v>
       </c>
       <c r="Y14">
-        <v>0.143</v>
+        <v>0.16</v>
       </c>
       <c r="Z14" t="s">
         <v>197</v>
       </c>
       <c r="AA14" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="AB14">
-        <v>12.1464997681966</v>
+        <v>15.7951107363978</v>
       </c>
       <c r="AC14">
-        <v>53699</v>
+        <v>60481</v>
       </c>
       <c r="AD14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE14">
-        <v>14.3</v>
+        <v>16</v>
       </c>
       <c r="AF14">
         <v>5</v>
@@ -2513,94 +2513,94 @@
         <v>45</v>
       </c>
       <c r="B15">
-        <v>17798</v>
+        <v>15337</v>
       </c>
       <c r="C15">
-        <v>8147</v>
+        <v>6621</v>
       </c>
       <c r="D15">
+        <v>4</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15">
+        <v>75</v>
+      </c>
+      <c r="N15">
+        <v>50</v>
+      </c>
+      <c r="O15">
+        <v>50</v>
+      </c>
+      <c r="P15">
+        <v>2.5</v>
+      </c>
+      <c r="Q15">
+        <v>8</v>
+      </c>
+      <c r="R15" t="s">
+        <v>108</v>
+      </c>
+      <c r="S15">
+        <v>3834</v>
+      </c>
+      <c r="T15">
+        <v>0</v>
+      </c>
+      <c r="U15" t="b">
+        <v>0</v>
+      </c>
+      <c r="V15" t="b">
+        <v>1</v>
+      </c>
+      <c r="W15">
         <v>5</v>
-      </c>
-      <c r="E15">
-        <v>0</v>
-      </c>
-      <c r="F15">
-        <v>1</v>
-      </c>
-      <c r="G15">
-        <v>3</v>
-      </c>
-      <c r="H15">
-        <v>0</v>
-      </c>
-      <c r="I15">
-        <v>0</v>
-      </c>
-      <c r="J15">
-        <v>0</v>
-      </c>
-      <c r="K15">
-        <v>1</v>
-      </c>
-      <c r="L15">
-        <v>4</v>
-      </c>
-      <c r="M15">
-        <v>100</v>
-      </c>
-      <c r="N15">
-        <v>20</v>
-      </c>
-      <c r="O15">
-        <v>80</v>
-      </c>
-      <c r="P15">
-        <v>4</v>
-      </c>
-      <c r="Q15">
-        <v>11</v>
-      </c>
-      <c r="R15" t="s">
-        <v>109</v>
-      </c>
-      <c r="S15">
-        <v>3560</v>
-      </c>
-      <c r="T15">
-        <v>20</v>
-      </c>
-      <c r="U15" t="b">
-        <v>0</v>
-      </c>
-      <c r="V15" t="b">
-        <v>1</v>
-      </c>
-      <c r="W15">
-        <v>4</v>
       </c>
       <c r="X15" t="s">
         <v>124</v>
       </c>
       <c r="Y15">
-        <v>0.237</v>
+        <v>0.195</v>
       </c>
       <c r="Z15" t="s">
         <v>198</v>
       </c>
       <c r="AA15" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="AB15">
-        <v>35.09875408544925</v>
+        <v>26.65128595503306</v>
       </c>
       <c r="AC15">
-        <v>33653.73333333333</v>
+        <v>42852.77777777778</v>
       </c>
       <c r="AD15">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="AE15">
-        <v>23.7</v>
+        <v>19.5</v>
       </c>
       <c r="AF15">
         <v>5</v>
@@ -2611,61 +2611,61 @@
         <v>46</v>
       </c>
       <c r="B16">
-        <v>3033</v>
+        <v>17798</v>
       </c>
       <c r="C16">
-        <v>1394</v>
+        <v>8147</v>
       </c>
       <c r="D16">
+        <v>5</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16">
+        <v>3</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="K16">
+        <v>1</v>
+      </c>
+      <c r="L16">
         <v>4</v>
-      </c>
-      <c r="E16">
-        <v>0</v>
-      </c>
-      <c r="F16">
-        <v>0</v>
-      </c>
-      <c r="G16">
-        <v>1</v>
-      </c>
-      <c r="H16">
-        <v>0</v>
-      </c>
-      <c r="I16">
-        <v>0</v>
-      </c>
-      <c r="J16">
-        <v>0</v>
-      </c>
-      <c r="K16">
-        <v>0</v>
-      </c>
-      <c r="L16">
-        <v>3</v>
       </c>
       <c r="M16">
         <v>100</v>
       </c>
       <c r="N16">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="O16">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="P16">
-        <v>3.75</v>
+        <v>4</v>
       </c>
       <c r="Q16">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="R16" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="S16">
-        <v>758</v>
+        <v>3560</v>
       </c>
       <c r="T16">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="U16" t="b">
         <v>0</v>
@@ -2674,13 +2674,13 @@
         <v>1</v>
       </c>
       <c r="W16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="X16" t="s">
         <v>125</v>
       </c>
       <c r="Y16">
-        <v>0.216</v>
+        <v>0.237</v>
       </c>
       <c r="Z16" t="s">
         <v>199</v>
@@ -2689,19 +2689,19 @@
         <v>268</v>
       </c>
       <c r="AB16">
-        <v>39.47179649750809</v>
+        <v>35.09875408544925</v>
       </c>
       <c r="AC16">
-        <v>33457</v>
+        <v>33653.73333333333</v>
       </c>
       <c r="AD16">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="AE16">
-        <v>21.6</v>
+        <v>23.7</v>
       </c>
       <c r="AF16">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:32">
@@ -2709,13 +2709,13 @@
         <v>47</v>
       </c>
       <c r="B17">
-        <v>1091</v>
+        <v>3033</v>
       </c>
       <c r="C17">
-        <v>473</v>
+        <v>1394</v>
       </c>
       <c r="D17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E17">
         <v>0</v>
@@ -2724,7 +2724,7 @@
         <v>0</v>
       </c>
       <c r="G17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17">
         <v>0</v>
@@ -2739,28 +2739,28 @@
         <v>0</v>
       </c>
       <c r="L17">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M17">
         <v>100</v>
       </c>
       <c r="N17">
-        <v>33.3</v>
+        <v>75</v>
       </c>
       <c r="O17">
-        <v>33.3</v>
+        <v>75</v>
       </c>
       <c r="P17">
-        <v>1.333333333333333</v>
+        <v>3.75</v>
       </c>
       <c r="Q17">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="R17" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="S17">
-        <v>364</v>
+        <v>758</v>
       </c>
       <c r="T17">
         <v>0</v>
@@ -2778,7 +2778,7 @@
         <v>126</v>
       </c>
       <c r="Y17">
-        <v>0.202</v>
+        <v>0.216</v>
       </c>
       <c r="Z17" t="s">
         <v>200</v>
@@ -2787,16 +2787,16 @@
         <v>269</v>
       </c>
       <c r="AB17">
-        <v>27.229997055395</v>
+        <v>39.47179649750809</v>
       </c>
       <c r="AC17">
-        <v>43331</v>
+        <v>33457</v>
       </c>
       <c r="AD17">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AE17">
-        <v>20.2</v>
+        <v>21.6</v>
       </c>
       <c r="AF17">
         <v>4</v>
@@ -2807,67 +2807,67 @@
         <v>48</v>
       </c>
       <c r="B18">
-        <v>259720</v>
+        <v>1091</v>
       </c>
       <c r="C18">
-        <v>119271</v>
+        <v>473</v>
       </c>
       <c r="D18">
-        <v>86</v>
+        <v>3</v>
       </c>
       <c r="E18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F18">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="H18">
         <v>0</v>
       </c>
       <c r="I18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K18">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="L18">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="M18">
-        <v>87.2</v>
+        <v>100</v>
       </c>
       <c r="N18">
-        <v>57</v>
+        <v>33.3</v>
       </c>
       <c r="O18">
-        <v>62.8</v>
+        <v>33.3</v>
       </c>
       <c r="P18">
-        <v>2.197674418604651</v>
+        <v>1.333333333333333</v>
       </c>
       <c r="Q18">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="R18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="S18">
-        <v>3020</v>
+        <v>364</v>
       </c>
       <c r="T18">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="U18" t="b">
         <v>0</v>
       </c>
       <c r="V18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W18">
         <v>3</v>
@@ -2876,7 +2876,7 @@
         <v>127</v>
       </c>
       <c r="Y18">
-        <v>0.14</v>
+        <v>0.202</v>
       </c>
       <c r="Z18" t="s">
         <v>201</v>
@@ -2885,19 +2885,19 @@
         <v>270</v>
       </c>
       <c r="AB18">
-        <v>17.26007516464241</v>
+        <v>27.229997055395</v>
       </c>
       <c r="AC18">
-        <v>68590.43093922651</v>
+        <v>43331</v>
       </c>
       <c r="AD18">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="AE18">
-        <v>14</v>
+        <v>20.2</v>
       </c>
       <c r="AF18">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:32">
@@ -2905,67 +2905,67 @@
         <v>49</v>
       </c>
       <c r="B19">
-        <v>281</v>
+        <v>259720</v>
       </c>
       <c r="C19">
-        <v>132</v>
+        <v>119271</v>
       </c>
       <c r="D19">
-        <v>1</v>
+        <v>86</v>
       </c>
       <c r="E19">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="G19">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="H19">
         <v>0</v>
       </c>
       <c r="I19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K19">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="L19">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="M19">
-        <v>100</v>
+        <v>87.2</v>
       </c>
       <c r="N19">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="O19">
-        <v>100</v>
+        <v>62.8</v>
       </c>
       <c r="P19">
-        <v>4</v>
+        <v>2.197674418604651</v>
       </c>
       <c r="Q19">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="R19" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="S19">
-        <v>281</v>
+        <v>3020</v>
       </c>
       <c r="T19">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="U19" t="b">
         <v>0</v>
       </c>
       <c r="V19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W19">
         <v>3</v>
@@ -2974,25 +2974,25 @@
         <v>128</v>
       </c>
       <c r="Y19">
-        <v>0.135</v>
+        <v>0.14</v>
       </c>
       <c r="Z19" t="s">
         <v>202</v>
       </c>
       <c r="AA19" t="s">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="AB19">
-        <v>8.32682799895915</v>
+        <v>17.26007516464241</v>
       </c>
       <c r="AC19">
-        <v>63849</v>
+        <v>68590.43093922651</v>
       </c>
       <c r="AD19">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="AE19">
-        <v>13.5</v>
+        <v>14</v>
       </c>
       <c r="AF19">
         <v>3</v>
@@ -3078,7 +3078,7 @@
         <v>203</v>
       </c>
       <c r="AA20" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="AB20">
         <v>15.55547228644085</v>
@@ -3274,7 +3274,7 @@
         <v>205</v>
       </c>
       <c r="AA22" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="AB22">
         <v>11.48220438684129</v>
@@ -3303,7 +3303,7 @@
         <v>33</v>
       </c>
       <c r="D23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23">
         <v>0</v>
@@ -3312,7 +3312,7 @@
         <v>0</v>
       </c>
       <c r="G23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H23">
         <v>0</v>
@@ -3327,7 +3327,7 @@
         <v>0</v>
       </c>
       <c r="L23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M23">
         <v>100</v>
@@ -3336,10 +3336,10 @@
         <v>100</v>
       </c>
       <c r="O23">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="P23">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="Q23">
         <v>9</v>
@@ -3348,7 +3348,7 @@
         <v>106</v>
       </c>
       <c r="S23">
-        <v>40</v>
+        <v>79</v>
       </c>
       <c r="T23">
         <v>0</v>
@@ -3372,7 +3372,7 @@
         <v>206</v>
       </c>
       <c r="AA23" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AB23">
         <v>3.53581142339075</v>
@@ -3470,7 +3470,7 @@
         <v>207</v>
       </c>
       <c r="AA24" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AB24">
         <v>33.55941432703644</v>
@@ -3493,22 +3493,22 @@
         <v>55</v>
       </c>
       <c r="B25">
-        <v>248</v>
+        <v>3260</v>
       </c>
       <c r="C25">
-        <v>122</v>
+        <v>1555</v>
       </c>
       <c r="D25">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="E25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F25">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G25">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H25">
         <v>0</v>
@@ -3520,34 +3520,34 @@
         <v>0</v>
       </c>
       <c r="K25">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L25">
         <v>2</v>
       </c>
       <c r="M25">
-        <v>66.7</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="N25">
-        <v>66.7</v>
+        <v>58.8</v>
       </c>
       <c r="O25">
-        <v>100</v>
+        <v>47.1</v>
       </c>
       <c r="P25">
-        <v>4</v>
+        <v>1.235294117647059</v>
       </c>
       <c r="Q25">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="R25" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="S25">
-        <v>83</v>
+        <v>192</v>
       </c>
       <c r="T25">
-        <v>0</v>
+        <v>11.8</v>
       </c>
       <c r="U25" t="b">
         <v>0</v>
@@ -3562,25 +3562,25 @@
         <v>134</v>
       </c>
       <c r="Y25">
-        <v>0.114</v>
+        <v>0.115</v>
       </c>
       <c r="Z25" t="s">
         <v>208</v>
       </c>
       <c r="AA25" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="AB25">
-        <v>20.7642596234897</v>
+        <v>10.56717274351188</v>
       </c>
       <c r="AC25">
-        <v>68450</v>
+        <v>71494.25</v>
       </c>
       <c r="AD25">
         <v>0</v>
       </c>
       <c r="AE25">
-        <v>11.4</v>
+        <v>11.5</v>
       </c>
       <c r="AF25">
         <v>3</v>
@@ -3591,13 +3591,13 @@
         <v>56</v>
       </c>
       <c r="B26">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C26">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="D26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26">
         <v>0</v>
@@ -3606,7 +3606,7 @@
         <v>0</v>
       </c>
       <c r="G26">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H26">
         <v>0</v>
@@ -3621,13 +3621,13 @@
         <v>0</v>
       </c>
       <c r="L26">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M26">
         <v>100</v>
       </c>
       <c r="N26">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="O26">
         <v>100</v>
@@ -3642,7 +3642,7 @@
         <v>106</v>
       </c>
       <c r="S26">
-        <v>249</v>
+        <v>124</v>
       </c>
       <c r="T26">
         <v>0</v>
@@ -3660,25 +3660,25 @@
         <v>135</v>
       </c>
       <c r="Y26">
-        <v>0.135</v>
+        <v>0.114</v>
       </c>
       <c r="Z26" t="s">
         <v>209</v>
       </c>
       <c r="AA26" t="s">
-        <v>257</v>
+        <v>276</v>
       </c>
       <c r="AB26">
-        <v>7.268578878748371</v>
+        <v>20.7642596234897</v>
       </c>
       <c r="AC26">
-        <v>57875</v>
+        <v>68450</v>
       </c>
       <c r="AD26">
         <v>0</v>
       </c>
       <c r="AE26">
-        <v>13.5</v>
+        <v>11.4</v>
       </c>
       <c r="AF26">
         <v>3</v>
@@ -3689,61 +3689,61 @@
         <v>57</v>
       </c>
       <c r="B27">
-        <v>3260</v>
+        <v>281</v>
       </c>
       <c r="C27">
-        <v>1555</v>
+        <v>132</v>
       </c>
       <c r="D27">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E27">
         <v>0</v>
       </c>
       <c r="F27">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+      <c r="L27">
+        <v>0</v>
+      </c>
+      <c r="M27">
+        <v>100</v>
+      </c>
+      <c r="N27">
+        <v>0</v>
+      </c>
+      <c r="O27">
+        <v>100</v>
+      </c>
+      <c r="P27">
         <v>4</v>
       </c>
-      <c r="H27">
-        <v>0</v>
-      </c>
-      <c r="I27">
-        <v>0</v>
-      </c>
-      <c r="J27">
-        <v>0</v>
-      </c>
-      <c r="K27">
-        <v>2</v>
-      </c>
-      <c r="L27">
-        <v>2</v>
-      </c>
-      <c r="M27">
-        <v>70.59999999999999</v>
-      </c>
-      <c r="N27">
-        <v>58.8</v>
-      </c>
-      <c r="O27">
-        <v>47.1</v>
-      </c>
-      <c r="P27">
-        <v>1.235294117647059</v>
-      </c>
       <c r="Q27">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="R27" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="S27">
-        <v>192</v>
+        <v>281</v>
       </c>
       <c r="T27">
-        <v>11.8</v>
+        <v>0</v>
       </c>
       <c r="U27" t="b">
         <v>0</v>
@@ -3758,25 +3758,25 @@
         <v>136</v>
       </c>
       <c r="Y27">
-        <v>0.115</v>
+        <v>0.135</v>
       </c>
       <c r="Z27" t="s">
         <v>210</v>
       </c>
       <c r="AA27" t="s">
-        <v>271</v>
+        <v>256</v>
       </c>
       <c r="AB27">
-        <v>10.56717274351188</v>
+        <v>8.32682799895915</v>
       </c>
       <c r="AC27">
-        <v>71494.25</v>
+        <v>63849</v>
       </c>
       <c r="AD27">
         <v>0</v>
       </c>
       <c r="AE27">
-        <v>11.5</v>
+        <v>13.5</v>
       </c>
       <c r="AF27">
         <v>3</v>
@@ -3862,7 +3862,7 @@
         <v>211</v>
       </c>
       <c r="AA28" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="AB28">
         <v>10.98200315956885</v>
@@ -3960,7 +3960,7 @@
         <v>189</v>
       </c>
       <c r="AA29" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="AB29">
         <v>9.88428158148505</v>
@@ -4058,7 +4058,7 @@
         <v>212</v>
       </c>
       <c r="AA30" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="AB30">
         <v>16.6188482216708</v>
@@ -4156,7 +4156,7 @@
         <v>213</v>
       </c>
       <c r="AA31" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="AB31">
         <v>22.9785145516815</v>
@@ -4254,7 +4254,7 @@
         <v>214</v>
       </c>
       <c r="AA32" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="AB32">
         <v>14.8293963254593</v>
@@ -4352,7 +4352,7 @@
         <v>215</v>
       </c>
       <c r="AA33" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="AB33">
         <v>20.36663306550204</v>
@@ -4447,10 +4447,10 @@
         <v>0.116</v>
       </c>
       <c r="Z34" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="AA34" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="AB34">
         <v>14.11904489235</v>
@@ -4646,7 +4646,7 @@
         <v>217</v>
       </c>
       <c r="AA36" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="AB36">
         <v>17.1103809315335</v>
@@ -4744,7 +4744,7 @@
         <v>218</v>
       </c>
       <c r="AA37" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="AB37">
         <v>15.51486597305606</v>
@@ -4842,7 +4842,7 @@
         <v>219</v>
       </c>
       <c r="AA38" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="AB38">
         <v>18.620890311318</v>
@@ -4940,7 +4940,7 @@
         <v>220</v>
       </c>
       <c r="AA39" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="AB39">
         <v>32.93807267950098</v>
@@ -4963,19 +4963,19 @@
         <v>70</v>
       </c>
       <c r="B40">
-        <v>2561</v>
+        <v>249</v>
       </c>
       <c r="C40">
-        <v>1271</v>
+        <v>115</v>
       </c>
       <c r="D40">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E40">
         <v>0</v>
       </c>
       <c r="F40">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G40">
         <v>0</v>
@@ -4987,7 +4987,7 @@
         <v>0</v>
       </c>
       <c r="J40">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K40">
         <v>0</v>
@@ -4999,22 +4999,22 @@
         <v>100</v>
       </c>
       <c r="N40">
+        <v>0</v>
+      </c>
+      <c r="O40">
         <v>100</v>
       </c>
-      <c r="O40">
-        <v>50</v>
-      </c>
       <c r="P40">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="Q40">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="R40" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="S40">
-        <v>1280</v>
+        <v>249</v>
       </c>
       <c r="T40">
         <v>0</v>
@@ -5023,7 +5023,7 @@
         <v>0</v>
       </c>
       <c r="V40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W40">
         <v>3</v>
@@ -5032,25 +5032,25 @@
         <v>149</v>
       </c>
       <c r="Y40">
-        <v>0.185</v>
+        <v>0.135</v>
       </c>
       <c r="Z40" t="s">
         <v>221</v>
       </c>
       <c r="AA40" t="s">
-        <v>286</v>
+        <v>257</v>
       </c>
       <c r="AB40">
-        <v>24.1636296257439</v>
+        <v>7.268578878748371</v>
       </c>
       <c r="AC40">
-        <v>46913.66666666666</v>
+        <v>57875</v>
       </c>
       <c r="AD40">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE40">
-        <v>18.5</v>
+        <v>13.5</v>
       </c>
       <c r="AF40">
         <v>3</v>
@@ -5136,7 +5136,7 @@
         <v>222</v>
       </c>
       <c r="AA41" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="AB41">
         <v>17.91530339429697</v>
@@ -5234,7 +5234,7 @@
         <v>223</v>
       </c>
       <c r="AA42" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="AB42">
         <v>37.48260738597017</v>
@@ -5528,7 +5528,7 @@
         <v>226</v>
       </c>
       <c r="AA45" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="AB45">
         <v>13.76209990809102</v>
@@ -5724,7 +5724,7 @@
         <v>228</v>
       </c>
       <c r="AA47" t="s">
-        <v>286</v>
+        <v>262</v>
       </c>
       <c r="AB47">
         <v>18.91913348477285</v>
@@ -5822,7 +5822,7 @@
         <v>229</v>
       </c>
       <c r="AA48" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="AB48">
         <v>11.70126280863145</v>
@@ -5949,10 +5949,10 @@
         <v>2570</v>
       </c>
       <c r="D50">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E50">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F50">
         <v>0</v>
@@ -5976,16 +5976,16 @@
         <v>2</v>
       </c>
       <c r="M50">
-        <v>75</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="N50">
-        <v>75</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="O50">
         <v>100</v>
       </c>
       <c r="P50">
-        <v>2.5</v>
+        <v>2.142857142857143</v>
       </c>
       <c r="Q50">
         <v>8</v>
@@ -5994,10 +5994,10 @@
         <v>108</v>
       </c>
       <c r="S50">
-        <v>723</v>
+        <v>826</v>
       </c>
       <c r="T50">
-        <v>25</v>
+        <v>28.6</v>
       </c>
       <c r="U50" t="b">
         <v>0</v>
@@ -6018,7 +6018,7 @@
         <v>231</v>
       </c>
       <c r="AA50" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="AB50">
         <v>10.47677697204727</v>
@@ -6407,7 +6407,7 @@
         <v>0.142</v>
       </c>
       <c r="Z54" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AA54" t="s">
         <v>291</v>
@@ -6508,7 +6508,7 @@
         <v>235</v>
       </c>
       <c r="AA55" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="AB55">
         <v>18.42384950637563</v>
@@ -6606,7 +6606,7 @@
         <v>236</v>
       </c>
       <c r="AA56" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="AB56">
         <v>9.86925565256</v>
@@ -6704,7 +6704,7 @@
         <v>237</v>
       </c>
       <c r="AA57" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="AB57">
         <v>13.21785906579786</v>
@@ -6929,7 +6929,7 @@
         <v>803</v>
       </c>
       <c r="D60">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E60">
         <v>0</v>
@@ -6938,7 +6938,7 @@
         <v>1</v>
       </c>
       <c r="G60">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H60">
         <v>0</v>
@@ -6953,19 +6953,19 @@
         <v>0</v>
       </c>
       <c r="L60">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M60">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="N60">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="O60">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="P60">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q60">
         <v>8</v>
@@ -6974,7 +6974,7 @@
         <v>108</v>
       </c>
       <c r="S60">
-        <v>350</v>
+        <v>438</v>
       </c>
       <c r="T60">
         <v>0</v>
@@ -7194,7 +7194,7 @@
         <v>241</v>
       </c>
       <c r="AA62" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="AB62">
         <v>20.3029065312299</v>
@@ -7684,7 +7684,7 @@
         <v>246</v>
       </c>
       <c r="AA67" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="AB67">
         <v>9.460431841561114</v>
@@ -7782,7 +7782,7 @@
         <v>247</v>
       </c>
       <c r="AA68" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="AB68">
         <v>26.46976704214084</v>
@@ -7978,7 +7978,7 @@
         <v>249</v>
       </c>
       <c r="AA70" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="AB70">
         <v>9.767140251129691</v>
@@ -8076,7 +8076,7 @@
         <v>250</v>
       </c>
       <c r="AA71" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="AB71">
         <v>8.876398510931251</v>
@@ -8174,7 +8174,7 @@
         <v>251</v>
       </c>
       <c r="AA72" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="AB72">
         <v>15.52107361214972</v>
@@ -8370,7 +8370,7 @@
         <v>253</v>
       </c>
       <c r="AA74" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="AB74">
         <v>14.38464784497463</v>

</xml_diff>

<commit_message>
Add SNAP CPP verification: snap_source column, verified hover/table labels
- Scraped Texas Community Partner Program (CPP) for all 74 MHM counties
  using toh=2 (SNAP enrollment assistance); found 157 unique orgs
- Cross-referenced against catalog with city-constrained fuzzy matching;
  15 sites upgraded from heuristic to "CPP verified"
- Added snap_source column to catalog: "CPP verified" (15), "heuristic" (68)
- Pantry map hover tooltip now shows "Yes (CPP verified)" vs plain "Yes"
- Results table SNAP Assist column reflects CPP verification status
- Saved cpp_snap_orgs.xlsx with full CPP org list for reference

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/food_access_county.xlsx
+++ b/food_access_county.xlsx
@@ -2929,7 +2929,7 @@
         <v>1</v>
       </c>
       <c r="J19">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K19">
         <v>12</v>
@@ -3419,7 +3419,7 @@
         <v>0</v>
       </c>
       <c r="J24">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K24">
         <v>3</v>
@@ -4889,7 +4889,7 @@
         <v>0</v>
       </c>
       <c r="J39">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K39">
         <v>1</v>
@@ -5085,7 +5085,7 @@
         <v>0</v>
       </c>
       <c r="J41">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K41">
         <v>0</v>
@@ -7535,7 +7535,7 @@
         <v>0</v>
       </c>
       <c r="J66">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K66">
         <v>2</v>
@@ -8319,7 +8319,7 @@
         <v>0</v>
       </c>
       <c r="J74">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="K74">
         <v>11</v>

</xml_diff>